<commit_message>
Enhance Google Drive integration and update environment configuration
- Added support for downloading Excel files from Google Drive and Google Sheets, allowing for dynamic configuration loading.
- Introduced new environment variables for Google Drive integration, including `GOOGLE_SHEET_URL` and `GOOGLE_DRIVE_FILE_ID`.
- Updated `.env.local` to include a new variable for a published Google Sheet URL.
- Created `GOOGLE_DRIVE_SETUP.md` for detailed instructions on configuring Google Drive and Sheets.
- Improved error handling and logging during the Excel file download process.
- Refactored the Excel loading logic to accommodate new download methods and ensure the latest data is always used.
- Updated README to reflect changes in environment variable usage and Google Drive requirements.
</commit_message>
<xml_diff>
--- a/storage/config.xlsx
+++ b/storage/config.xlsx
@@ -7,15 +7,13 @@
     <sheet sheetId="1" name="sources" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="filters" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="notifications" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="sent" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="schedules" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="45">
   <si>
     <t>id</t>
   </si>
@@ -50,6 +48,12 @@
     <t>https://remaxrd.com/propiedades?businessTypes=sale&amp;currencyType=us&amp;locations[]=id-440%26description-BAYAHIBE%26&amp;typeProperty[]=apartment&amp;ciudad=BAYAHIBE</t>
   </si>
   <si>
+    <t>TRUE</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
     <t>page</t>
   </si>
   <si>
@@ -68,6 +72,9 @@
     <t>https://c21sunsets.com/es/s/bayahibe-la-altagracia</t>
   </si>
   <si>
+    <t>10</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -95,6 +102,9 @@
     <t>textMustExclude</t>
   </si>
   <si>
+    <t>160000</t>
+  </si>
+  <si>
     <t>República Dominicana</t>
   </si>
   <si>
@@ -138,27 +148,6 @@
   </si>
   <si>
     <t>Encontramos {{count}} nuevas propiedades</t>
-  </si>
-  <si>
-    <t>listingId</t>
-  </si>
-  <si>
-    <t>hash</t>
-  </si>
-  <si>
-    <t>notifiedAt</t>
-  </si>
-  <si>
-    <t>cron</t>
-  </si>
-  <si>
-    <t>timezone</t>
-  </si>
-  <si>
-    <t>0 14 * * *</t>
-  </si>
-  <si>
-    <t>America/Santo_Domingo</t>
   </si>
 </sst>
 </file>
@@ -537,14 +526,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="80" customWidth="1"/>
-    <col min="4" max="5" width="10" customWidth="1"/>
-    <col min="6" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="15" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -582,46 +563,46 @@
       <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="D2" t="b">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" t="s">
+      <c r="H3" t="s">
         <v>15</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" t="b">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>10</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" t="s">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -634,64 +615,57 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="6" width="10" customWidth="1"/>
-    <col min="7" max="8" width="30" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="H1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2">
-        <v>500000</v>
+      <c r="A2" t="s">
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="D2" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2">
-        <v>2</v>
-      </c>
-      <c r="F2">
-        <v>2</v>
+        <v>32</v>
+      </c>
+      <c r="E2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F2" t="s">
+        <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -704,121 +678,45 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="50" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="6" width="50" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D2">
-        <v>10</v>
+        <v>42</v>
+      </c>
+      <c r="D2" t="s">
+        <v>19</v>
       </c>
       <c r="E2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="F2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="50" customWidth="1"/>
-    <col min="4" max="4" width="25" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" t="s">
         <v>44</v>
-      </c>
-      <c r="C1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C2" t="s">
-        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement AI market analysis and enhance property listing features
- Introduced AI-driven market analysis functionality using Groq, allowing for insights on property listings.
- Updated .env.local to include new AI configuration variables such as GROQ_API_KEY and AI_MODEL.
- Enhanced property data structure to include AI analysis results, providing actionable insights for listings.
- Updated email rendering to display AI analysis summaries and visual indicators for opportunities and alerts.
- Added new scripts for analyzing property data and integrated AI analysis into the scraping process.
- Improved README documentation to reflect new AI features and usage instructions.
</commit_message>
<xml_diff>
--- a/storage/config.xlsx
+++ b/storage/config.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
   <si>
     <t>id</t>
   </si>
@@ -102,7 +102,7 @@
     <t>textMustExclude</t>
   </si>
   <si>
-    <t>500000</t>
+    <t>160000</t>
   </si>
   <si>
     <t>República Dominicana</t>
@@ -135,10 +135,7 @@
     <t>whatsappTemplate</t>
   </si>
   <si>
-    <t>tu-email@gmail.com,otro-email@example.com</t>
-  </si>
-  <si>
-    <t>+1234567890,+0987654321</t>
+    <t>agus.massaing@gmail.com</t>
   </si>
   <si>
     <t>14:00</t>
@@ -704,19 +701,19 @@
         <v>40</v>
       </c>
       <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s">
         <v>41</v>
-      </c>
-      <c r="C2" t="s">
-        <v>42</v>
       </c>
       <c r="D2" t="s">
         <v>19</v>
       </c>
       <c r="E2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F2" t="s">
         <v>43</v>
-      </c>
-      <c r="F2" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>